<commit_message>
Sync from .app 5064c13: Ukrainian estimate page (/uk/), Norwegian copy, phone hero order, tablet tooltip fix
- tools/sync-from-app.sh mirrors uk/ like pl/ (canonical .eu, sign-up and legal on .app)
- sitemap.xml now lists /uk/koshtorys-elektromontazhni-roboty/

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/downloads/tilbudsmal-elektriker.xlsx
+++ b/site/downloads/tilbudsmal-elektriker.xlsx
@@ -604,17 +604,17 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Ikke MVA-registrert? Slett MVA-linjen og «MVA» bak org.nr.</t>
+          <t>Ikke MVA-registrert? Sett satsen til 0 % og fjern «MVA» etter org.nr.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Pris (Fastpris / Prisoverslag):</t>
+          <t>Pristype:</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
     </row>
-    <row r="7">
+    <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>KUNDE</t>
@@ -622,7 +622,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>ADRESSE FOR ARBEIDET (hvis annen)</t>
+          <t>OPPDRAGSADRESSE (hvis en annen enn kundens)</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>[Beskriv nøyaktig hva du skal gjøre.]</t>
+          <t>[Velg fastpris eller prisoverslag i feltet Pristype. Beskriv omfang, materialer, forutsetninger og avtalt oppstart og ferdigstillelse.]</t>
         </is>
       </c>
     </row>
@@ -707,9 +707,8 @@
       <c r="B19" s="12" t="n"/>
       <c r="C19" s="12" t="n"/>
       <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13">
+      <c r="E19" s="13" t="str">
         <f>IF(OR(B19="",D19=""),"",B19*D19)</f>
-        <v/>
       </c>
     </row>
     <row r="20">
@@ -717,9 +716,8 @@
       <c r="B20" s="12" t="n"/>
       <c r="C20" s="12" t="n"/>
       <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13">
+      <c r="E20" s="13" t="str">
         <f>IF(OR(B20="",D20=""),"",B20*D20)</f>
-        <v/>
       </c>
     </row>
     <row r="21">
@@ -727,9 +725,8 @@
       <c r="B21" s="12" t="n"/>
       <c r="C21" s="12" t="n"/>
       <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13">
+      <c r="E21" s="13" t="str">
         <f>IF(OR(B21="",D21=""),"",B21*D21)</f>
-        <v/>
       </c>
     </row>
     <row r="22">
@@ -737,9 +734,8 @@
       <c r="B22" s="12" t="n"/>
       <c r="C22" s="12" t="n"/>
       <c r="D22" s="13" t="n"/>
-      <c r="E22" s="13">
+      <c r="E22" s="13" t="str">
         <f>IF(OR(B22="",D22=""),"",B22*D22)</f>
-        <v/>
       </c>
     </row>
     <row r="23">
@@ -747,9 +743,8 @@
       <c r="B23" s="12" t="n"/>
       <c r="C23" s="12" t="n"/>
       <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13">
+      <c r="E23" s="13" t="str">
         <f>IF(OR(B23="",D23=""),"",B23*D23)</f>
-        <v/>
       </c>
     </row>
     <row r="24">
@@ -757,9 +752,8 @@
       <c r="B24" s="12" t="n"/>
       <c r="C24" s="12" t="n"/>
       <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13">
+      <c r="E24" s="13" t="str">
         <f>IF(OR(B24="",D24=""),"",B24*D24)</f>
-        <v/>
       </c>
     </row>
     <row r="26">
@@ -801,9 +795,8 @@
       <c r="B28" s="12" t="n"/>
       <c r="C28" s="12" t="n"/>
       <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13">
+      <c r="E28" s="13" t="str">
         <f>IF(OR(B28="",D28=""),"",B28*D28)</f>
-        <v/>
       </c>
     </row>
     <row r="29">
@@ -811,9 +804,8 @@
       <c r="B29" s="12" t="n"/>
       <c r="C29" s="12" t="n"/>
       <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13">
+      <c r="E29" s="13" t="str">
         <f>IF(OR(B29="",D29=""),"",B29*D29)</f>
-        <v/>
       </c>
     </row>
     <row r="30">
@@ -821,9 +813,8 @@
       <c r="B30" s="12" t="n"/>
       <c r="C30" s="12" t="n"/>
       <c r="D30" s="13" t="n"/>
-      <c r="E30" s="13">
+      <c r="E30" s="13" t="str">
         <f>IF(OR(B30="",D30=""),"",B30*D30)</f>
-        <v/>
       </c>
     </row>
     <row r="31">
@@ -831,9 +822,8 @@
       <c r="B31" s="12" t="n"/>
       <c r="C31" s="12" t="n"/>
       <c r="D31" s="13" t="n"/>
-      <c r="E31" s="13">
+      <c r="E31" s="13" t="str">
         <f>IF(OR(B31="",D31=""),"",B31*D31)</f>
-        <v/>
       </c>
     </row>
     <row r="32">
@@ -841,9 +831,8 @@
       <c r="B32" s="12" t="n"/>
       <c r="C32" s="12" t="n"/>
       <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13">
+      <c r="E32" s="13" t="str">
         <f>IF(OR(B32="",D32=""),"",B32*D32)</f>
-        <v/>
       </c>
     </row>
     <row r="33">
@@ -851,9 +840,8 @@
       <c r="B33" s="12" t="n"/>
       <c r="C33" s="12" t="n"/>
       <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13">
+      <c r="E33" s="13" t="str">
         <f>IF(OR(B33="",D33=""),"",B33*D33)</f>
-        <v/>
       </c>
     </row>
     <row r="35">
@@ -874,12 +862,12 @@
     <row r="36">
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Sum eks. MVA</t>
-        </is>
-      </c>
-      <c r="E36" s="13">
+          <t>Sum ekskl. MVA</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="n">
         <f>SUM(E19:E24)+SUM(E28:E33)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -888,20 +876,20 @@
           <t>MVA</t>
         </is>
       </c>
-      <c r="E37" s="13">
+      <c r="E37" s="13" t="n">
         <f>ROUND(E36*D35,2)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>TOTALT</t>
-        </is>
-      </c>
-      <c r="E38" s="16">
+          <t>TOTALT Å BETALE</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="n">
         <f>E36+E37</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -914,7 +902,7 @@
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>Bygningsmessige arbeider som hulltaking og utbedring av overflater (puss, maling), feil i den eksisterende installasjonen og gebyrer fra nettselskapet – hvis dette ikke er nevnt over. Tilleggsarbeid prises separat før det starter.</t>
+          <t>Med mindre annet er oppgitt, er hulltaking, overflatearbeid, utbedring av feil i eksisterende anlegg og gebyrer fra nettselskapet ikke inkludert. Tilleggsarbeid og pris avtales før arbeidet starter.</t>
         </is>
       </c>
     </row>
@@ -928,7 +916,7 @@
     <row r="44" ht="26" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Samsvarserklæring og annen dokumentasjon som gjelder arbeidet leveres til eieren av anlegget, der det er aktuelt – senest ved ferdigstillelse, eller sammen med fakturaen for små oppdrag.</t>
+          <t>Påkrevd samsvarserklæring og tilhørende dokumentasjon leveres til anleggseieren ved ferdigstillelse.</t>
         </is>
       </c>
     </row>
@@ -942,7 +930,7 @@
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>Forskudd [__] % ved aksept. Resten betales innen [__] dager etter ferdigstillelse.</t>
+          <t>Eventuelt avtalt forskudd: [__] %. Restbeløpet forfaller [__] dager etter ferdigstillelse.</t>
         </is>
       </c>
     </row>
@@ -963,7 +951,7 @@
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="17" t="inlineStr">
         <is>
-          <t>Tilbudet er gyldig i 30 dager fra datoen over.</t>
+          <t>Tilbudet gjelder til datoen i feltet «Gyldig til».</t>
         </is>
       </c>
     </row>
@@ -974,10 +962,10 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="15" customHeight="1">
+    <row r="53" ht="26" customHeight="1">
       <c r="A53" s="17" t="inlineStr">
         <is>
-          <t>Jeg aksepterer dette tilbudet og vilkårene over.</t>
+          <t>Jeg godtar tilbudet og vilkårene ovenfor. Avtalen begrenser ikke forbrukerens lovfestede rettigheter.</t>
         </is>
       </c>
     </row>
@@ -1008,7 +996,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="A50:E50"/>
@@ -1021,6 +1009,7 @@
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A44:E44"/>
     <mergeCell ref="A13:E15"/>
+    <mergeCell ref="C7:E7"/>
   </mergeCells>
   <pageMargins left="0.6" right="0.6" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>